<commit_message>
Convert JSON files from LFS to normal Git New dist & time matrix
</commit_message>
<xml_diff>
--- a/docs/路線最佳化比較結果.xlsx
+++ b/docs/路線最佳化比較結果.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeff0\OneDrive\桌面\115_NTUT_Thesis\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFECEB4-E6CB-4F84-88E9-EF997CD5CFEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A589EAB5-0C4A-4FB9-B0A9-744C34766826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10070" xr2:uid="{BFA22242-4AF4-4033-990C-8B00A20BC4F2}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="38730" windowHeight="21210" xr2:uid="{BFA22242-4AF4-4033-990C-8B00A20BC4F2}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="7">
   <si>
     <t>vehicle num</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -209,9 +209,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -222,6 +219,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -558,39 +558,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80168C42-45BC-48F9-BA8B-850284450034}">
-  <dimension ref="A1:O39"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:O47"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.453125" customWidth="1"/>
-    <col min="2" max="3" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.453125" customWidth="1"/>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="2" max="3" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
-      <c r="B1" s="12">
+      <c r="B1" s="16">
         <v>45994</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12">
+      <c r="C1" s="16"/>
+      <c r="D1" s="16">
         <v>45996</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12">
+      <c r="E1" s="16"/>
+      <c r="F1" s="16">
         <v>45998</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12">
+      <c r="G1" s="16"/>
+      <c r="H1" s="16">
         <v>45999</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12">
+      <c r="I1" s="16"/>
+      <c r="J1" s="16">
         <v>46000</v>
       </c>
-      <c r="K1" s="12"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -623,7 +623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -658,7 +658,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -693,7 +693,7 @@
         <v>3253.42</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -728,7 +728,7 @@
         <v>268.97000000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -763,7 +763,7 @@
         <v>0.87</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -798,30 +798,30 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="13">
+      <c r="B9" s="12">
         <v>46001</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="13">
+      <c r="C9" s="13"/>
+      <c r="D9" s="12">
         <v>46003</v>
       </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="13">
+      <c r="E9" s="13"/>
+      <c r="F9" s="12">
         <v>46004</v>
       </c>
-      <c r="G9" s="14"/>
-      <c r="H9" s="13">
+      <c r="G9" s="13"/>
+      <c r="H9" s="12">
         <v>46005</v>
       </c>
-      <c r="I9" s="14"/>
-      <c r="J9" s="13">
+      <c r="I9" s="13"/>
+      <c r="J9" s="12">
         <v>46006</v>
       </c>
-      <c r="K9" s="14"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K9" s="13"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>4</v>
@@ -854,7 +854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
@@ -889,7 +889,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>2</v>
       </c>
@@ -924,7 +924,7 @@
         <v>3106.47</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
@@ -959,7 +959,7 @@
         <v>263.72000000000003</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>5</v>
       </c>
@@ -994,7 +994,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>6</v>
       </c>
@@ -1029,30 +1029,30 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="13">
+      <c r="B17" s="12">
         <v>46007</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="13">
+      <c r="C17" s="13"/>
+      <c r="D17" s="12">
         <v>46008</v>
       </c>
-      <c r="E17" s="14"/>
-      <c r="F17" s="13">
+      <c r="E17" s="13"/>
+      <c r="F17" s="12">
         <v>46010</v>
       </c>
-      <c r="G17" s="14"/>
-      <c r="H17" s="13">
+      <c r="G17" s="13"/>
+      <c r="H17" s="12">
         <v>46011</v>
       </c>
-      <c r="I17" s="14"/>
-      <c r="J17" s="13">
+      <c r="I17" s="13"/>
+      <c r="J17" s="12">
         <v>46012</v>
       </c>
-      <c r="K17" s="14"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="K17" s="13"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
         <v>4</v>
@@ -1085,7 +1085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>2</v>
       </c>
@@ -1155,7 +1155,7 @@
         <v>3425.42</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>3</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>276.19</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>6</v>
       </c>
@@ -1260,18 +1260,18 @@
         <v>0.93</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="13">
+      <c r="B25" s="12">
         <v>46013</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="13">
+      <c r="C25" s="13"/>
+      <c r="D25" s="12">
         <v>46014</v>
       </c>
-      <c r="E25" s="14"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="E25" s="13"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
         <v>4</v>
@@ -1286,7 +1286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>0</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>2</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>4424.2700000000004</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>3</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>308.45999999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>5</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>0.92</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>6</v>
       </c>
@@ -1371,38 +1371,38 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="13">
+      <c r="B33" s="12">
         <v>46018</v>
       </c>
-      <c r="C33" s="14"/>
-      <c r="D33" s="13">
+      <c r="C33" s="13"/>
+      <c r="D33" s="12">
         <v>46021</v>
       </c>
-      <c r="E33" s="14"/>
-      <c r="F33" s="13">
+      <c r="E33" s="13"/>
+      <c r="F33" s="12">
         <v>46022</v>
       </c>
-      <c r="G33" s="14"/>
-      <c r="H33" s="13">
+      <c r="G33" s="13"/>
+      <c r="H33" s="12">
         <v>45659</v>
       </c>
-      <c r="I33" s="14"/>
-      <c r="J33" s="15">
+      <c r="I33" s="13"/>
+      <c r="J33" s="14">
         <v>45663</v>
       </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="13">
+      <c r="K33" s="15"/>
+      <c r="L33" s="12">
         <v>45664</v>
       </c>
-      <c r="M33" s="14"/>
-      <c r="N33" s="13">
+      <c r="M33" s="13"/>
+      <c r="N33" s="12">
         <v>45670</v>
       </c>
-      <c r="O33" s="14"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="O33" s="13"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
         <v>4</v>
@@ -1447,7 +1447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>0</v>
       </c>
@@ -1494,7 +1494,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>2</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>3253.84</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>3</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>268.43</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>5</v>
       </c>
@@ -1635,7 +1635,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>6</v>
       </c>
@@ -1682,8 +1682,172 @@
         <v>0.97</v>
       </c>
     </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="B41" s="12">
+        <v>46024</v>
+      </c>
+      <c r="C41" s="13"/>
+      <c r="D41" s="12">
+        <v>46028</v>
+      </c>
+      <c r="E41" s="13"/>
+      <c r="F41" s="12">
+        <v>46031</v>
+      </c>
+      <c r="G41" s="13"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B43" s="6">
+        <v>136</v>
+      </c>
+      <c r="C43" s="3">
+        <v>105</v>
+      </c>
+      <c r="D43" s="6">
+        <v>159</v>
+      </c>
+      <c r="E43" s="3">
+        <v>131</v>
+      </c>
+      <c r="F43" s="6">
+        <v>94</v>
+      </c>
+      <c r="G43" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B44" s="7">
+        <v>5483.61</v>
+      </c>
+      <c r="C44" s="5">
+        <v>4677.76</v>
+      </c>
+      <c r="D44" s="7">
+        <v>6875.32</v>
+      </c>
+      <c r="E44" s="5">
+        <v>5774.84</v>
+      </c>
+      <c r="F44" s="7">
+        <v>4151.9799999999996</v>
+      </c>
+      <c r="G44" s="5">
+        <v>4059.06</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B45" s="6">
+        <v>353.62</v>
+      </c>
+      <c r="C45" s="3">
+        <v>331.56</v>
+      </c>
+      <c r="D45" s="6">
+        <v>398.14</v>
+      </c>
+      <c r="E45" s="3">
+        <v>368.05</v>
+      </c>
+      <c r="F45" s="6">
+        <v>310.88</v>
+      </c>
+      <c r="G45" s="3">
+        <v>309.06</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B46" s="2">
+        <v>0.68</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0.87</v>
+      </c>
+      <c r="D46" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0.91</v>
+      </c>
+      <c r="F46" s="2">
+        <v>0.79</v>
+      </c>
+      <c r="G46" s="3">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="C47" s="3">
+        <v>0.96</v>
+      </c>
+      <c r="D47" s="2">
+        <v>0.94</v>
+      </c>
+      <c r="E47" s="3">
+        <v>0.99</v>
+      </c>
+      <c r="F47" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="G47" s="6">
+        <v>0.95</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="27">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:K9"/>
     <mergeCell ref="N33:O33"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="D25:E25"/>
@@ -1698,16 +1862,6 @@
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="F33:G33"/>
     <mergeCell ref="H33:I33"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>